<commit_message>
Additionnal details for RDRAM controlled impedance
</commit_message>
<xml_diff>
--- a/Required_impedance_control.xlsx
+++ b/Required_impedance_control.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Timéo\Desktop\Matterhorn 64\GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{317657C7-4CAC-4A0B-9097-FD4E27C60DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE471D69-3471-4E04-AF01-B79014BF1FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="2730" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="7" r:id="rId1"/>
@@ -65,12 +65,39 @@
         </r>
       </text>
     </comment>
+    <comment ref="D3" authorId="0" shapeId="0" xr:uid="{D4B2A778-FB0B-4E52-970E-3307E9F2A9B7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="宋体"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Administrator:
+4 options：</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="宋体"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+Differential Pair (Non coplanar)
+Differential Pair (Coplanar)
+Single Ended (Non coplanar)
+Single Ended (Coplanar)
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="40">
   <si>
     <t>Reference Layer</t>
   </si>
@@ -129,57 +156,212 @@
     <t>Both Top and Bottom Layers</t>
   </si>
   <si>
-    <t>Please contact me in case something isn't clear.</t>
-  </si>
-  <si>
     <t xml:space="preserve">The traces wich require the controlled impedance are selected, and are highlighted in white. </t>
   </si>
   <si>
-    <t>Rambus Dynamic RAM
+    <t>Single Ended (Coplanar)</t>
+  </si>
+  <si>
+    <t>Trace Width (mils)</t>
+  </si>
+  <si>
+    <t>23.24 mils (0.5903 mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please consider that both top layer (Layer 1) and bottom layer (Layer 4) contain traces that require 50 Ohms of impedance. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">This curved trace requires  22 Ohms of
+impedance. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best regards. </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Rambus Dynamic RAM
+Data Traces TOP LAYER
+(RDRAM)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TOP LAYER</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Rambus Dynamic RAM
 Data Traces
-(RDRAM)</t>
-  </si>
-  <si>
-    <t>Single Ended (Non Coplanar)</t>
-  </si>
-  <si>
-    <t>Single Ended (Coplanar)</t>
-  </si>
-  <si>
-    <t>Trace Width (mils)</t>
-  </si>
-  <si>
-    <t>23.24 mils (0.5903 mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Please consider that both top layer (Layer 1) and bottom layer (Layer 4) contain traces that require 50 Ohms of impedance. </t>
-  </si>
-  <si>
-    <t>Required stackup: JLC04161H-3313
+(RDRAM)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>BOTTOM LAYER</t>
+    </r>
+  </si>
+  <si>
+    <t>L4</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <r>
+      <t>Single Ended (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Non Coplanar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Single Ended (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Coplanar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>6.06 mils (0.1539 mm)</t>
+  </si>
+  <si>
+    <t>Since the bottom traces are coplanar, their width are a bit smaller (6.06 mils instead of the 6.16 mils used on top).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Please take a look at the calculation screenshot bellow. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feel free to reach out if something isn't clear. </t>
+  </si>
+  <si>
+    <t>RDRAM TOP LAYER CALCULATION</t>
+  </si>
+  <si>
+    <t>RDRAM BOTTOM LAYER CALCULATION</t>
+  </si>
+  <si>
+    <t>CCTLPGM CALCULATION</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Required stackup: JLC04161H-3313
 All the selected layers (in white)
 require 50 Ohms of impedance. 
 Please take a look at the more detailed pictures bellow. 
+The TOP traces are single ended </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>non coplanar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, but the BOTTOM traces are </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>coplanar.
+Calculations screenshot are available bellow.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 Feel free to reach out in case you need to confirm something. 
 Thanks a lot!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">This curved trace requires  22 Ohms of
-impedance. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Best regards. </t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="13">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -226,6 +408,37 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -247,7 +460,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -387,45 +600,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -434,20 +656,29 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,13 +702,13 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>81643</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>56518</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2971553</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>3</xdr:row>
       <xdr:rowOff>2452854</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -514,16 +745,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>125786</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>49103</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1395655</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>23929</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2763792</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>23930</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -602,15 +833,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>244929</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>2924074</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>2785529</xdr:colOff>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>108858</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -646,15 +877,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2707820</xdr:colOff>
-      <xdr:row>7</xdr:row>
+      <xdr:row>9</xdr:row>
       <xdr:rowOff>285749</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>2701688</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>3481006</xdr:colOff>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -680,6 +911,182 @@
         <a:xfrm>
           <a:off x="8477249" y="6300106"/>
           <a:ext cx="6293975" cy="4204608"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>58615</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>219808</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>3019176</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>2194081</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Image 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14115DAE-4CCA-487E-B78C-B63926349753}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18317307" y="2725616"/>
+          <a:ext cx="2960561" cy="1974273"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>53</xdr:row>
+      <xdr:rowOff>121227</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1322302</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>34989</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Image 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F25CB8D-75E9-91B7-31B9-0CF16E79F52C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="18166772"/>
+          <a:ext cx="13393075" cy="4104762"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>173182</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1300655</xdr:colOff>
+      <xdr:row>99</xdr:row>
+      <xdr:rowOff>58372</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Image 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7883733E-9A13-B7FB-0FF5-EA1643E4DBC7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="23033182"/>
+          <a:ext cx="13371428" cy="4076190"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>54</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>30443</xdr:colOff>
+      <xdr:row>75</xdr:row>
+      <xdr:rowOff>95822</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Image 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0AC9B79F-3DE0-F000-4B5B-F5F6E8C34EB5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15230475" y="18440400"/>
+          <a:ext cx="13384493" cy="4096322"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -949,7 +1356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.5703125" customWidth="1"/>
@@ -977,7 +1384,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>9</v>
@@ -993,8 +1400,8 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="174.75" customHeight="1">
-      <c r="A2" s="33" t="s">
-        <v>21</v>
+      <c r="A2" s="32" t="s">
+        <v>26</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>6</v>
@@ -1003,7 +1410,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>7</v>
@@ -1015,283 +1422,327 @@
         <v>50</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="9" t="s">
-        <v>27</v>
+      <c r="I2" s="34" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="198" customHeight="1">
       <c r="A3" s="32" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>10</v>
       </c>
       <c r="G3" s="7">
+        <v>50</v>
+      </c>
+      <c r="I3" s="33"/>
+    </row>
+    <row r="4" spans="1:9" ht="252" customHeight="1">
+      <c r="A4" s="31" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1"/>
-    <row r="6" spans="1:9" ht="23.25">
-      <c r="B6" s="10" t="s">
+      <c r="F4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="7">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" thickBot="1"/>
+    <row r="8" spans="1:9" ht="23.25">
+      <c r="A8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12"/>
-    </row>
-    <row r="7" spans="1:9" ht="23.25">
-      <c r="B7" s="13" t="s">
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="12"/>
+    </row>
+    <row r="9" spans="1:9" ht="23.25">
+      <c r="A9" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14" t="s">
+      <c r="B9" s="14"/>
+      <c r="C9" s="14"/>
+      <c r="D9" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14" t="s">
+      <c r="E9" s="14"/>
+      <c r="F9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="15"/>
-    </row>
-    <row r="8" spans="1:9" ht="23.25">
-      <c r="B8" s="13"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="15"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="B9" s="16"/>
-      <c r="H9" s="17"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="B10" s="16"/>
-      <c r="H10" s="17"/>
+      <c r="G9" s="15"/>
+    </row>
+    <row r="10" spans="1:9" ht="23.25">
+      <c r="A10" s="13"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="15"/>
     </row>
     <row r="11" spans="1:9">
-      <c r="B11" s="16"/>
-      <c r="H11" s="17"/>
+      <c r="A11" s="16"/>
+      <c r="G11" s="17"/>
     </row>
     <row r="12" spans="1:9">
-      <c r="B12" s="16"/>
-      <c r="H12" s="17"/>
+      <c r="A12" s="16"/>
+      <c r="G12" s="17"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="B13" s="16"/>
-      <c r="H13" s="17"/>
+      <c r="A13" s="16"/>
+      <c r="G13" s="17"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="B14" s="16"/>
-      <c r="H14" s="17"/>
+      <c r="A14" s="16"/>
+      <c r="G14" s="17"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="B15" s="16"/>
-      <c r="H15" s="17"/>
+      <c r="A15" s="16"/>
+      <c r="G15" s="17"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="B16" s="16"/>
-      <c r="H16" s="17"/>
-    </row>
-    <row r="17" spans="2:8">
-      <c r="B17" s="16"/>
-      <c r="H17" s="17"/>
-    </row>
-    <row r="18" spans="2:8">
-      <c r="B18" s="16"/>
-      <c r="H18" s="17"/>
-    </row>
-    <row r="19" spans="2:8">
-      <c r="B19" s="16"/>
-      <c r="H19" s="17"/>
-    </row>
-    <row r="20" spans="2:8">
-      <c r="B20" s="16"/>
-      <c r="H20" s="17"/>
-    </row>
-    <row r="21" spans="2:8">
-      <c r="B21" s="16"/>
-      <c r="H21" s="17"/>
-    </row>
-    <row r="22" spans="2:8">
-      <c r="B22" s="16"/>
-      <c r="H22" s="17"/>
-    </row>
-    <row r="23" spans="2:8">
-      <c r="B23" s="16"/>
-      <c r="H23" s="17"/>
-    </row>
-    <row r="24" spans="2:8">
-      <c r="B24" s="16"/>
-      <c r="H24" s="17"/>
-    </row>
-    <row r="25" spans="2:8">
-      <c r="B25" s="16"/>
-      <c r="H25" s="17"/>
-    </row>
-    <row r="26" spans="2:8">
-      <c r="B26" s="16"/>
-      <c r="H26" s="17"/>
-    </row>
-    <row r="27" spans="2:8">
-      <c r="B27" s="16"/>
-      <c r="H27" s="17"/>
-    </row>
-    <row r="28" spans="2:8">
-      <c r="B28" s="16"/>
-      <c r="H28" s="17"/>
-    </row>
-    <row r="29" spans="2:8">
-      <c r="B29" s="16"/>
-      <c r="H29" s="17"/>
-    </row>
-    <row r="30" spans="2:8">
-      <c r="B30" s="16"/>
-      <c r="H30" s="17"/>
-    </row>
-    <row r="31" spans="2:8">
-      <c r="B31" s="16"/>
-      <c r="H31" s="17"/>
-    </row>
-    <row r="32" spans="2:8">
-      <c r="B32" s="16"/>
-      <c r="H32" s="17"/>
-    </row>
-    <row r="33" spans="2:8">
-      <c r="B33" s="16"/>
-      <c r="H33" s="17"/>
-    </row>
-    <row r="34" spans="2:8">
-      <c r="B34" s="16"/>
-      <c r="H34" s="17"/>
-    </row>
-    <row r="35" spans="2:8" ht="15.75" thickBot="1">
-      <c r="B35" s="16"/>
-      <c r="H35" s="17"/>
-    </row>
-    <row r="36" spans="2:8">
-      <c r="B36" s="16"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="22"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="17"/>
-    </row>
-    <row r="37" spans="2:8" ht="23.25">
-      <c r="B37" s="16"/>
-      <c r="E37" s="24" t="s">
+      <c r="A16" s="16"/>
+      <c r="G16" s="17"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="16"/>
+      <c r="G17" s="17"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="16"/>
+      <c r="G18" s="17"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="16"/>
+      <c r="G19" s="17"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="16"/>
+      <c r="G20" s="17"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="16"/>
+      <c r="G21" s="17"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="16"/>
+      <c r="G22" s="17"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="16"/>
+      <c r="G23" s="17"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="16"/>
+      <c r="G24" s="17"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="16"/>
+      <c r="G25" s="17"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="16"/>
+      <c r="G26" s="17"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="16"/>
+      <c r="G27" s="17"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="16"/>
+      <c r="G28" s="17"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="16"/>
+      <c r="G29" s="17"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="16"/>
+      <c r="G30" s="17"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="16"/>
+      <c r="G31" s="17"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="16"/>
+      <c r="G32" s="17"/>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="16"/>
+      <c r="G33" s="17"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="16"/>
+      <c r="G34" s="17"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="16"/>
+      <c r="G35" s="17"/>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="16"/>
+      <c r="G36" s="17"/>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A37" s="16"/>
+      <c r="G37" s="17"/>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="16"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="23"/>
+      <c r="G38" s="17"/>
+    </row>
+    <row r="39" spans="1:7" ht="23.25">
+      <c r="A39" s="16"/>
+      <c r="D39" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="F37" s="25"/>
-      <c r="G37" s="26"/>
-      <c r="H37" s="17"/>
-    </row>
-    <row r="38" spans="2:8">
-      <c r="B38" s="16"/>
-      <c r="E38" s="27" t="s">
-        <v>26</v>
-      </c>
-      <c r="F38" s="25"/>
-      <c r="G38" s="26"/>
-      <c r="H38" s="17"/>
-    </row>
-    <row r="39" spans="2:8">
-      <c r="B39" s="16"/>
-      <c r="E39" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="F39" s="25"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="17"/>
-    </row>
-    <row r="40" spans="2:8">
-      <c r="B40" s="16"/>
-      <c r="E40" s="28"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="26"/>
-      <c r="H40" s="17"/>
-    </row>
-    <row r="41" spans="2:8">
-      <c r="B41" s="16"/>
-      <c r="E41" s="27" t="s">
+      <c r="E39" s="25"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="17"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="16"/>
+      <c r="D40" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="E40" s="25"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="17"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="16"/>
+      <c r="D41" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F41" s="25"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="17"/>
-    </row>
-    <row r="42" spans="2:8">
-      <c r="B42" s="16"/>
-      <c r="E42" s="27" t="s">
-        <v>29</v>
-      </c>
-      <c r="F42" s="25"/>
-      <c r="G42" s="26"/>
-      <c r="H42" s="17"/>
-    </row>
-    <row r="43" spans="2:8">
-      <c r="B43" s="16"/>
-      <c r="E43" s="28"/>
-      <c r="F43" s="25"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="17"/>
-    </row>
-    <row r="44" spans="2:8">
-      <c r="B44" s="16"/>
-      <c r="E44" s="28"/>
-      <c r="F44" s="25"/>
-      <c r="G44" s="26"/>
-      <c r="H44" s="17"/>
-    </row>
-    <row r="45" spans="2:8" ht="15.75" thickBot="1">
-      <c r="B45" s="16"/>
-      <c r="E45" s="29"/>
-      <c r="F45" s="30"/>
-      <c r="G45" s="31"/>
-      <c r="H45" s="17"/>
-    </row>
-    <row r="46" spans="2:8">
-      <c r="B46" s="16"/>
-      <c r="H46" s="17"/>
-    </row>
-    <row r="47" spans="2:8">
-      <c r="B47" s="16"/>
-      <c r="H47" s="17"/>
-    </row>
-    <row r="48" spans="2:8">
-      <c r="B48" s="16"/>
-      <c r="H48" s="17"/>
-    </row>
-    <row r="49" spans="2:8" ht="15.75" thickBot="1">
-      <c r="B49" s="18"/>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="20"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="17"/>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="16"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="26"/>
+      <c r="G42" s="17"/>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="16"/>
+      <c r="D43" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="E43" s="25"/>
+      <c r="F43" s="26"/>
+      <c r="G43" s="17"/>
+    </row>
+    <row r="44" spans="1:7">
+      <c r="A44" s="16"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="25"/>
+      <c r="F44" s="26"/>
+      <c r="G44" s="17"/>
+    </row>
+    <row r="45" spans="1:7">
+      <c r="A45" s="16"/>
+      <c r="D45" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="E45" s="25"/>
+      <c r="F45" s="26"/>
+      <c r="G45" s="17"/>
+    </row>
+    <row r="46" spans="1:7">
+      <c r="A46" s="16"/>
+      <c r="D46" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="E46" s="25"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="17"/>
+    </row>
+    <row r="47" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A47" s="16"/>
+      <c r="D47" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="E47" s="29"/>
+      <c r="F47" s="30"/>
+      <c r="G47" s="17"/>
+    </row>
+    <row r="48" spans="1:7">
+      <c r="A48" s="16"/>
+      <c r="G48" s="17"/>
+    </row>
+    <row r="49" spans="1:7">
+      <c r="A49" s="16"/>
+      <c r="G49" s="17"/>
+    </row>
+    <row r="50" spans="1:7">
+      <c r="A50" s="16"/>
+      <c r="G50" s="17"/>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" thickBot="1">
+      <c r="A51" s="18"/>
+      <c r="B51" s="19"/>
+      <c r="C51" s="19"/>
+      <c r="D51" s="19"/>
+      <c r="E51" s="19"/>
+      <c r="F51" s="19"/>
+      <c r="G51" s="20"/>
+    </row>
+    <row r="53" spans="1:7" ht="33.75">
+      <c r="A53" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="G53" s="38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" ht="31.5">
+      <c r="A77" s="38" t="s">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I2:I3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>